<commit_message>
in gstr1 report add credit note
</commit_message>
<xml_diff>
--- a/src/templates/GSTR-1.xlsx
+++ b/src/templates/GSTR-1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="b2b" sheetId="1" state="visible" r:id="rId2"/>
@@ -17,6 +17,7 @@
     <sheet name="at" sheetId="7" state="visible" r:id="rId8"/>
     <sheet name="hsn(b2b)" sheetId="8" state="visible" r:id="rId9"/>
     <sheet name="hsn(b2c)" sheetId="9" state="visible" r:id="rId10"/>
+    <sheet name="docs" sheetId="10" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="66">
   <si>
     <t xml:space="preserve">Summary For B2B(4)</t>
   </si>
@@ -205,6 +206,27 @@
   </si>
   <si>
     <t xml:space="preserve">State/UT Tax Amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary of documents issued during the tax period (13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Cancelled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nature of Document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sr. No. From</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sr. No. To</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancelled</t>
   </si>
 </sst>
 </file>
@@ -402,7 +424,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -549,6 +571,14 @@
     </xf>
     <xf numFmtId="165" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -630,13 +660,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M4"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="19.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.04"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -740,19 +770,87 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="17.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.01"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="84.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13.36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -840,11 +938,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.04"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -922,17 +1020,17 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N4"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="17.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="23.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="5.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="19.35"/>
@@ -1052,14 +1150,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="23.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="5.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="19.35"/>
@@ -1161,7 +1259,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.74"/>
@@ -1265,11 +1363,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.04"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1333,7 +1431,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6.01"/>
@@ -1342,7 +1440,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="5.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="21.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.1"/>
   </cols>
@@ -1473,7 +1571,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6.01"/>
@@ -1482,7 +1580,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="5.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="21.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.1"/>
   </cols>

</xml_diff>